<commit_message>
Actualizando datos con complementos a entrega 3 en siguiente sesión
</commit_message>
<xml_diff>
--- a/df_total_e3.xlsx
+++ b/df_total_e3.xlsx
@@ -963,7 +963,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>4.1</t>
+          <t>4.8</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -982,7 +982,7 @@
         </is>
       </c>
       <c r="G12" t="n">
-        <v>4.057142857142857</v>
+        <v>4.776785714285714</v>
       </c>
       <c r="H12" t="inlineStr">
         <is>
@@ -1008,12 +1008,12 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>3.8</t>
+          <t>4.8</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -1023,12 +1023,12 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>E3.Func_B</t>
+          <t>E3.Func_A</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>Existe exploración morfológica pero con menor toma de riesgos. La escala es adecuada en general. El manejo de la topografía es funcional (cumple con niveles) pero carece de una intención poética o de integración profunda con el código.</t>
+          <t>Las 5 propuestas demuestran una exploración morfológica arriesgada y diversa. El manejo de la escala es impecable. La propuesta integra la topografía del lote de forma creativa, convirtiendo la pendiente en una oportunidad proyectual.</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
@@ -1055,12 +1055,12 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>3.0</t>
+          <t>4.5</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
@@ -1070,12 +1070,12 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>E3.Rep_B</t>
+          <t>E3.Rep_A</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>La representación técnica es legible pero carece de detalles esenciales (ej. falta de cotas o amoblamiento genérico que no explica el uso). La factura de las maquetas es aceptable, aunque se observan descuidos en la limpieza o su relación con la planimetría correspondiente</t>
+          <t>La planimetría (plantas 1:100) es clara, técnica y expresiva; incluye cotas, amoblamiento y una relación clara con el contexto/lote. Las maquetas volumétricas poseen una factura impecable y tienen relación directa con la planimetría correspondiente</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
@@ -1102,7 +1102,7 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>4.4</t>
+          <t>4.9</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -2136,7 +2136,7 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>4.6</t>
+          <t>4.9</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
@@ -2155,7 +2155,7 @@
         </is>
       </c>
       <c r="G37" t="n">
-        <v>4.628571428571429</v>
+        <v>4.901785714285714</v>
       </c>
       <c r="H37" t="inlineStr">
         <is>
@@ -2181,12 +2181,12 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>3.8</t>
+          <t>4.8</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
@@ -2196,12 +2196,12 @@
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>E3.Func_B</t>
+          <t>E3.Func_A</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>Existe exploración morfológica pero con menor toma de riesgos. La escala es adecuada en general. El manejo de la topografía es funcional (cumple con niveles) pero carece de una intención poética o de integración profunda con el código.</t>
+          <t>Las 5 propuestas demuestran una exploración morfológica arriesgada y diversa. El manejo de la escala es impecable. La propuesta integra la topografía del lote de forma creativa, convirtiendo la pendiente en una oportunidad proyectual.</t>
         </is>
       </c>
       <c r="H38" t="inlineStr">
@@ -2275,7 +2275,7 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>4.7</t>
+          <t>4.9</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
@@ -3310,7 +3310,7 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>4.6</t>
+          <t>4.8</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
@@ -3329,7 +3329,7 @@
         </is>
       </c>
       <c r="G62" t="n">
-        <v>4.575</v>
+        <v>4.81875</v>
       </c>
       <c r="H62" t="inlineStr">
         <is>
@@ -3355,12 +3355,12 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>3.9</t>
+          <t>4.9</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
@@ -3370,12 +3370,12 @@
       </c>
       <c r="F63" t="inlineStr">
         <is>
-          <t>E3.Func_B</t>
+          <t>E3.Func_A</t>
         </is>
       </c>
       <c r="G63" t="inlineStr">
         <is>
-          <t>Existe exploración morfológica pero con menor toma de riesgos. La escala es adecuada en general. El manejo de la topografía es funcional (cumple con niveles) pero carece de una intención poética o de integración profunda con el código.</t>
+          <t>Las 5 propuestas demuestran una exploración morfológica arriesgada y diversa. El manejo de la escala es impecable. La propuesta integra la topografía del lote de forma creativa, convirtiendo la pendiente en una oportunidad proyectual.</t>
         </is>
       </c>
       <c r="H63" t="inlineStr">
@@ -5659,7 +5659,7 @@
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>4.5</t>
+          <t>4.7</t>
         </is>
       </c>
       <c r="D112" t="inlineStr">
@@ -5678,7 +5678,7 @@
         </is>
       </c>
       <c r="G112" t="n">
-        <v>4.516071428571429</v>
+        <v>4.741071428571429</v>
       </c>
       <c r="H112" t="inlineStr">
         <is>
@@ -5704,12 +5704,12 @@
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>3.6</t>
+          <t>4.5</t>
         </is>
       </c>
       <c r="D113" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="E113" t="inlineStr">
@@ -5719,12 +5719,12 @@
       </c>
       <c r="F113" t="inlineStr">
         <is>
-          <t>E3.Func_B</t>
+          <t>E3.Func_A</t>
         </is>
       </c>
       <c r="G113" t="inlineStr">
         <is>
-          <t>Existe exploración morfológica pero con menor toma de riesgos. La escala es adecuada en general. El manejo de la topografía es funcional (cumple con niveles) pero carece de una intención poética o de integración profunda con el código.</t>
+          <t>Las 5 propuestas demuestran una exploración morfológica arriesgada y diversa. El manejo de la escala es impecable. La propuesta integra la topografía del lote de forma creativa, convirtiendo la pendiente en una oportunidad proyectual.</t>
         </is>
       </c>
       <c r="H113" t="inlineStr">
@@ -6812,7 +6812,7 @@
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>3.3</t>
+          <t>3.5</t>
         </is>
       </c>
       <c r="D137" t="inlineStr">
@@ -6831,7 +6831,7 @@
         </is>
       </c>
       <c r="G137" t="n">
-        <v>3.2625</v>
+        <v>3.4625</v>
       </c>
       <c r="H137" t="inlineStr">
         <is>
@@ -6855,12 +6855,12 @@
       </c>
       <c r="C138" t="inlineStr">
         <is>
-          <t>3.2</t>
+          <t>4.0</t>
         </is>
       </c>
       <c r="D138" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="E138" t="inlineStr">
@@ -6870,12 +6870,12 @@
       </c>
       <c r="F138" t="inlineStr">
         <is>
-          <t>E3.Func_B</t>
+          <t>E3.Func_A</t>
         </is>
       </c>
       <c r="G138" t="inlineStr">
         <is>
-          <t>Existe exploración morfológica pero con menor toma de riesgos. La escala es adecuada en general. El manejo de la topografía es funcional (cumple con niveles) pero carece de una intención poética o de integración profunda con el código.</t>
+          <t>Las 5 propuestas demuestran una exploración morfológica arriesgada y diversa. El manejo de la escala es impecable. La propuesta integra la topografía del lote de forma creativa, convirtiendo la pendiente en una oportunidad proyectual.</t>
         </is>
       </c>
       <c r="H138" t="inlineStr">
@@ -7958,7 +7958,7 @@
       </c>
       <c r="C162" t="inlineStr">
         <is>
-          <t>4.0</t>
+          <t>4.2</t>
         </is>
       </c>
       <c r="D162" t="inlineStr">
@@ -7977,7 +7977,7 @@
         </is>
       </c>
       <c r="G162" t="n">
-        <v>4.010714285714286</v>
+        <v>4.198214285714286</v>
       </c>
       <c r="H162" t="inlineStr">
         <is>
@@ -8003,7 +8003,7 @@
       </c>
       <c r="C163" t="inlineStr">
         <is>
-          <t>3.0</t>
+          <t>3.8</t>
         </is>
       </c>
       <c r="D163" t="inlineStr">
@@ -9134,7 +9134,7 @@
       </c>
       <c r="C187" t="inlineStr">
         <is>
-          <t>4.8</t>
+          <t>5.0</t>
         </is>
       </c>
       <c r="D187" t="inlineStr">
@@ -9153,7 +9153,7 @@
         </is>
       </c>
       <c r="G187" t="n">
-        <v>4.75</v>
+        <v>5</v>
       </c>
       <c r="H187" t="inlineStr">
         <is>
@@ -9179,7 +9179,7 @@
       </c>
       <c r="C188" t="inlineStr">
         <is>
-          <t>4.0</t>
+          <t>5.0</t>
         </is>
       </c>
       <c r="D188" t="inlineStr">
@@ -10308,7 +10308,7 @@
       </c>
       <c r="C212" t="inlineStr">
         <is>
-          <t>4.8</t>
+          <t>5.0</t>
         </is>
       </c>
       <c r="D212" t="inlineStr">
@@ -10327,7 +10327,7 @@
         </is>
       </c>
       <c r="G212" t="n">
-        <v>4.75</v>
+        <v>5</v>
       </c>
       <c r="H212" t="inlineStr">
         <is>
@@ -10353,7 +10353,7 @@
       </c>
       <c r="C213" t="inlineStr">
         <is>
-          <t>4.0</t>
+          <t>5.0</t>
         </is>
       </c>
       <c r="D213" t="inlineStr">
@@ -11484,7 +11484,7 @@
       </c>
       <c r="C237" t="inlineStr">
         <is>
-          <t>1.4</t>
+          <t>2.7</t>
         </is>
       </c>
       <c r="D237" t="inlineStr">
@@ -11503,7 +11503,7 @@
         </is>
       </c>
       <c r="G237" t="n">
-        <v>1.422857142857143</v>
+        <v>2.698214285714286</v>
       </c>
       <c r="H237" t="inlineStr">
         <is>
@@ -11529,12 +11529,12 @@
       </c>
       <c r="C238" t="inlineStr">
         <is>
-          <t>2.0</t>
+          <t>3.4</t>
         </is>
       </c>
       <c r="D238" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>B</t>
         </is>
       </c>
       <c r="E238" t="inlineStr">
@@ -11544,12 +11544,12 @@
       </c>
       <c r="F238" t="inlineStr">
         <is>
-          <t>E3.Func_C</t>
+          <t>E3.Func_B</t>
         </is>
       </c>
       <c r="G238" t="inlineStr">
         <is>
-          <t>Escasa diversidad formal. Errores críticos de escala. La propuesta ignora la topografía o se limita a soluciones genéricas (ej. aplanamiento masivo) sin diálogo con el terreno.</t>
+          <t>Existe exploración morfológica pero con menor toma de riesgos. La escala es adecuada en general. El manejo de la topografía es funcional (cumple con niveles) pero carece de una intención poética o de integración profunda con el código.</t>
         </is>
       </c>
       <c r="H238" t="inlineStr">
@@ -11576,12 +11576,12 @@
       </c>
       <c r="C239" t="inlineStr">
         <is>
-          <t>2.1</t>
+          <t>3.2</t>
         </is>
       </c>
       <c r="D239" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>B</t>
         </is>
       </c>
       <c r="E239" t="inlineStr">
@@ -11591,12 +11591,12 @@
       </c>
       <c r="F239" t="inlineStr">
         <is>
-          <t>E3.Rep_C</t>
+          <t>E3.Rep_B</t>
         </is>
       </c>
       <c r="G239" t="inlineStr">
         <is>
-          <t>Planimetría confusa, incompleta o sin rigor técnico (falta de escala gráfica/numérica, linderos ausentes). Las maquetas son precarias y no permiten entender la espacialidad propuesta.</t>
+          <t>La representación técnica es legible pero carece de detalles esenciales (ej. falta de cotas o amoblamiento genérico que no explica el uso). La factura de las maquetas es aceptable, aunque se observan descuidos en la limpieza o su relación con la planimetría correspondiente</t>
         </is>
       </c>
       <c r="H239" t="inlineStr">
@@ -11623,12 +11623,12 @@
       </c>
       <c r="C240" t="inlineStr">
         <is>
-          <t>0.6</t>
+          <t>3.1</t>
         </is>
       </c>
       <c r="D240" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>B</t>
         </is>
       </c>
       <c r="E240" t="inlineStr">
@@ -11638,12 +11638,12 @@
       </c>
       <c r="F240" t="inlineStr">
         <is>
-          <t>E3.Arg_C</t>
+          <t>E3.Arg_B</t>
         </is>
       </c>
       <c r="G240" t="inlineStr">
         <is>
-          <t>La bitácora se presenta como un requisito administrativo y no como una herramienta de diseño. No hay coherencia entre el programa construido y las plantas presentadas. Faltan varios productos esenciales de la entrega.</t>
+          <t>La bitácora contiene los elementos solicitados, pero el vínculo entre el análisis (árbol, línea del tiempo, tabla y código) y las propuestas finales se siente forzado o desconectado. Hacen falta algunos productos.</t>
         </is>
       </c>
       <c r="H240" t="inlineStr">
@@ -12637,12 +12637,12 @@
       </c>
       <c r="C262" t="inlineStr">
         <is>
-          <t>3.5</t>
+          <t>4.5</t>
         </is>
       </c>
       <c r="D262" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="E262" t="inlineStr">
@@ -12652,11 +12652,11 @@
       </c>
       <c r="F262" t="inlineStr">
         <is>
-          <t>E3.Coment_B</t>
+          <t>E3.Coment_A</t>
         </is>
       </c>
       <c r="G262" t="n">
-        <v>3.46</v>
+        <v>4.494642857142857</v>
       </c>
       <c r="H262" t="inlineStr">
         <is>
@@ -12680,12 +12680,12 @@
       </c>
       <c r="C263" t="inlineStr">
         <is>
-          <t>2.8</t>
+          <t>4.6</t>
         </is>
       </c>
       <c r="D263" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>A</t>
         </is>
       </c>
       <c r="E263" t="inlineStr">
@@ -12695,12 +12695,12 @@
       </c>
       <c r="F263" t="inlineStr">
         <is>
-          <t>E3.Func_C</t>
+          <t>E3.Func_A</t>
         </is>
       </c>
       <c r="G263" t="inlineStr">
         <is>
-          <t>Escasa diversidad formal. Errores críticos de escala. La propuesta ignora la topografía o se limita a soluciones genéricas (ej. aplanamiento masivo) sin diálogo con el terreno.</t>
+          <t>Las 5 propuestas demuestran una exploración morfológica arriesgada y diversa. El manejo de la escala es impecable. La propuesta integra la topografía del lote de forma creativa, convirtiendo la pendiente en una oportunidad proyectual.</t>
         </is>
       </c>
       <c r="H263" t="inlineStr">
@@ -12725,12 +12725,12 @@
       </c>
       <c r="C264" t="inlineStr">
         <is>
-          <t>2.2</t>
+          <t>4.2</t>
         </is>
       </c>
       <c r="D264" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>A</t>
         </is>
       </c>
       <c r="E264" t="inlineStr">
@@ -12740,12 +12740,12 @@
       </c>
       <c r="F264" t="inlineStr">
         <is>
-          <t>E3.Rep_C</t>
+          <t>E3.Rep_A</t>
         </is>
       </c>
       <c r="G264" t="inlineStr">
         <is>
-          <t>Planimetría confusa, incompleta o sin rigor técnico (falta de escala gráfica/numérica, linderos ausentes). Las maquetas son precarias y no permiten entender la espacialidad propuesta.</t>
+          <t>La planimetría (plantas 1:100) es clara, técnica y expresiva; incluye cotas, amoblamiento y una relación clara con el contexto/lote. Las maquetas volumétricas poseen una factura impecable y tienen relación directa con la planimetría correspondiente</t>
         </is>
       </c>
       <c r="H264" t="inlineStr">
@@ -12770,7 +12770,7 @@
       </c>
       <c r="C265" t="inlineStr">
         <is>
-          <t>4.0</t>
+          <t>4.4</t>
         </is>
       </c>
       <c r="D265" t="inlineStr">
@@ -13783,12 +13783,12 @@
       </c>
       <c r="C287" t="inlineStr">
         <is>
-          <t>3.7</t>
+          <t>4.3</t>
         </is>
       </c>
       <c r="D287" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="E287" t="inlineStr">
@@ -13798,11 +13798,11 @@
       </c>
       <c r="F287" t="inlineStr">
         <is>
-          <t>E3.Coment_B</t>
+          <t>E3.Coment_A</t>
         </is>
       </c>
       <c r="G287" t="n">
-        <v>3.746428571428571</v>
+        <v>4.346428571428572</v>
       </c>
       <c r="H287" t="inlineStr">
         <is>
@@ -13828,12 +13828,12 @@
       </c>
       <c r="C288" t="inlineStr">
         <is>
-          <t>3.2</t>
+          <t>4.0</t>
         </is>
       </c>
       <c r="D288" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="E288" t="inlineStr">
@@ -13843,12 +13843,12 @@
       </c>
       <c r="F288" t="inlineStr">
         <is>
-          <t>E3.Func_B</t>
+          <t>E3.Func_A</t>
         </is>
       </c>
       <c r="G288" t="inlineStr">
         <is>
-          <t>Existe exploración morfológica pero con menor toma de riesgos. La escala es adecuada en general. El manejo de la topografía es funcional (cumple con niveles) pero carece de una intención poética o de integración profunda con el código.</t>
+          <t>Las 5 propuestas demuestran una exploración morfológica arriesgada y diversa. El manejo de la escala es impecable. La propuesta integra la topografía del lote de forma creativa, convirtiendo la pendiente en una oportunidad proyectual.</t>
         </is>
       </c>
       <c r="H288" t="inlineStr">
@@ -13875,12 +13875,12 @@
       </c>
       <c r="C289" t="inlineStr">
         <is>
-          <t>2.5</t>
+          <t>4.1</t>
         </is>
       </c>
       <c r="D289" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>A</t>
         </is>
       </c>
       <c r="E289" t="inlineStr">
@@ -13890,12 +13890,12 @@
       </c>
       <c r="F289" t="inlineStr">
         <is>
-          <t>E3.Rep_C</t>
+          <t>E3.Rep_A</t>
         </is>
       </c>
       <c r="G289" t="inlineStr">
         <is>
-          <t>Planimetría confusa, incompleta o sin rigor técnico (falta de escala gráfica/numérica, linderos ausentes). Las maquetas son precarias y no permiten entender la espacialidad propuesta.</t>
+          <t>La planimetría (plantas 1:100) es clara, técnica y expresiva; incluye cotas, amoblamiento y una relación clara con el contexto/lote. Las maquetas volumétricas poseen una factura impecable y tienen relación directa con la planimetría correspondiente</t>
         </is>
       </c>
       <c r="H289" t="inlineStr">
@@ -14957,7 +14957,7 @@
       </c>
       <c r="C312" t="inlineStr">
         <is>
-          <t>1.8</t>
+          <t>2.4</t>
         </is>
       </c>
       <c r="D312" t="inlineStr">
@@ -14976,7 +14976,7 @@
         </is>
       </c>
       <c r="G312" t="n">
-        <v>1.788571428571429</v>
+        <v>2.41875</v>
       </c>
       <c r="H312" t="inlineStr">
         <is>
@@ -15002,12 +15002,12 @@
       </c>
       <c r="C313" t="inlineStr">
         <is>
-          <t>2.9</t>
+          <t>3.7</t>
         </is>
       </c>
       <c r="D313" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>B</t>
         </is>
       </c>
       <c r="E313" t="inlineStr">
@@ -15017,12 +15017,12 @@
       </c>
       <c r="F313" t="inlineStr">
         <is>
-          <t>E3.Func_C</t>
+          <t>E3.Func_B</t>
         </is>
       </c>
       <c r="G313" t="inlineStr">
         <is>
-          <t>Escasa diversidad formal. Errores críticos de escala. La propuesta ignora la topografía o se limita a soluciones genéricas (ej. aplanamiento masivo) sin diálogo con el terreno.</t>
+          <t>Existe exploración morfológica pero con menor toma de riesgos. La escala es adecuada en general. El manejo de la topografía es funcional (cumple con niveles) pero carece de una intención poética o de integración profunda con el código.</t>
         </is>
       </c>
       <c r="H313" t="inlineStr">
@@ -15096,7 +15096,7 @@
       </c>
       <c r="C315" t="inlineStr">
         <is>
-          <t>0.7</t>
+          <t>2.5</t>
         </is>
       </c>
       <c r="D315" t="inlineStr">
@@ -16131,7 +16131,7 @@
       </c>
       <c r="C337" t="inlineStr">
         <is>
-          <t>4.0</t>
+          <t>4.2</t>
         </is>
       </c>
       <c r="D337" t="inlineStr">
@@ -16150,7 +16150,7 @@
         </is>
       </c>
       <c r="G337" t="n">
-        <v>3.988214285714286</v>
+        <v>4.179464285714285</v>
       </c>
       <c r="H337" t="inlineStr">
         <is>
@@ -16176,7 +16176,7 @@
       </c>
       <c r="C338" t="inlineStr">
         <is>
-          <t>3.1</t>
+          <t>3.8</t>
         </is>
       </c>
       <c r="D338" t="inlineStr">
@@ -17281,7 +17281,7 @@
       </c>
       <c r="C362" t="inlineStr">
         <is>
-          <t>4.4</t>
+          <t>4.8</t>
         </is>
       </c>
       <c r="D362" t="inlineStr">
@@ -17300,7 +17300,7 @@
         </is>
       </c>
       <c r="G362" t="n">
-        <v>4.357142857142858</v>
+        <v>4.834821428571429</v>
       </c>
       <c r="H362" t="inlineStr">
         <is>
@@ -17324,12 +17324,12 @@
       </c>
       <c r="C363" t="inlineStr">
         <is>
-          <t>3.0</t>
+          <t>4.6</t>
         </is>
       </c>
       <c r="D363" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="E363" t="inlineStr">
@@ -17339,12 +17339,12 @@
       </c>
       <c r="F363" t="inlineStr">
         <is>
-          <t>E3.Func_B</t>
+          <t>E3.Func_A</t>
         </is>
       </c>
       <c r="G363" t="inlineStr">
         <is>
-          <t>Existe exploración morfológica pero con menor toma de riesgos. La escala es adecuada en general. El manejo de la topografía es funcional (cumple con niveles) pero carece de una intención poética o de integración profunda con el código.</t>
+          <t>Las 5 propuestas demuestran una exploración morfológica arriesgada y diversa. El manejo de la escala es impecable. La propuesta integra la topografía del lote de forma creativa, convirtiendo la pendiente en una oportunidad proyectual.</t>
         </is>
       </c>
       <c r="H363" t="inlineStr">
@@ -17414,7 +17414,7 @@
       </c>
       <c r="C365" t="inlineStr">
         <is>
-          <t>4.4</t>
+          <t>4.7</t>
         </is>
       </c>
       <c r="D365" t="inlineStr">
@@ -18427,7 +18427,7 @@
       </c>
       <c r="C387" t="inlineStr">
         <is>
-          <t>4.7</t>
+          <t>5.0</t>
         </is>
       </c>
       <c r="D387" t="inlineStr">
@@ -18446,7 +18446,7 @@
         </is>
       </c>
       <c r="G387" t="n">
-        <v>4.734999999999999</v>
+        <v>4.98125</v>
       </c>
       <c r="H387" t="inlineStr">
         <is>
@@ -18472,12 +18472,12 @@
       </c>
       <c r="C388" t="inlineStr">
         <is>
-          <t>3.9</t>
+          <t>4.9</t>
         </is>
       </c>
       <c r="D388" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="E388" t="inlineStr">
@@ -18487,12 +18487,12 @@
       </c>
       <c r="F388" t="inlineStr">
         <is>
-          <t>E3.Func_B</t>
+          <t>E3.Func_A</t>
         </is>
       </c>
       <c r="G388" t="inlineStr">
         <is>
-          <t>Existe exploración morfológica pero con menor toma de riesgos. La escala es adecuada en general. El manejo de la topografía es funcional (cumple con niveles) pero carece de una intención poética o de integración profunda con el código.</t>
+          <t>Las 5 propuestas demuestran una exploración morfológica arriesgada y diversa. El manejo de la escala es impecable. La propuesta integra la topografía del lote de forma creativa, convirtiendo la pendiente en una oportunidad proyectual.</t>
         </is>
       </c>
       <c r="H388" t="inlineStr">
@@ -19582,12 +19582,12 @@
       </c>
       <c r="C412" t="inlineStr">
         <is>
-          <t>3.9</t>
+          <t>4.1</t>
         </is>
       </c>
       <c r="D412" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="E412" t="inlineStr">
@@ -19597,11 +19597,11 @@
       </c>
       <c r="F412" t="inlineStr">
         <is>
-          <t>E3.Coment_B</t>
+          <t>E3.Coment_A</t>
         </is>
       </c>
       <c r="G412" t="n">
-        <v>3.947857142857143</v>
+        <v>4.117857142857143</v>
       </c>
       <c r="H412" t="inlineStr">
         <is>
@@ -19625,12 +19625,12 @@
       </c>
       <c r="C413" t="inlineStr">
         <is>
-          <t>2.7</t>
+          <t>3.4</t>
         </is>
       </c>
       <c r="D413" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>B</t>
         </is>
       </c>
       <c r="E413" t="inlineStr">
@@ -19640,12 +19640,12 @@
       </c>
       <c r="F413" t="inlineStr">
         <is>
-          <t>E3.Func_C</t>
+          <t>E3.Func_B</t>
         </is>
       </c>
       <c r="G413" t="inlineStr">
         <is>
-          <t>Escasa diversidad formal. Errores críticos de escala. La propuesta ignora la topografía o se limita a soluciones genéricas (ej. aplanamiento masivo) sin diálogo con el terreno.</t>
+          <t>Existe exploración morfológica pero con menor toma de riesgos. La escala es adecuada en general. El manejo de la topografía es funcional (cumple con niveles) pero carece de una intención poética o de integración profunda con el código.</t>
         </is>
       </c>
       <c r="H413" t="inlineStr">
@@ -20727,7 +20727,7 @@
       </c>
       <c r="C437" t="inlineStr">
         <is>
-          <t>4.7</t>
+          <t>4.9</t>
         </is>
       </c>
       <c r="D437" t="inlineStr">
@@ -20746,7 +20746,7 @@
         </is>
       </c>
       <c r="G437" t="n">
-        <v>4.689285714285715</v>
+        <v>4.933035714285714</v>
       </c>
       <c r="H437" t="inlineStr">
         <is>
@@ -20772,12 +20772,12 @@
       </c>
       <c r="C438" t="inlineStr">
         <is>
-          <t>3.9</t>
+          <t>4.9</t>
         </is>
       </c>
       <c r="D438" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="E438" t="inlineStr">
@@ -20787,12 +20787,12 @@
       </c>
       <c r="F438" t="inlineStr">
         <is>
-          <t>E3.Func_B</t>
+          <t>E3.Func_A</t>
         </is>
       </c>
       <c r="G438" t="inlineStr">
         <is>
-          <t>Existe exploración morfológica pero con menor toma de riesgos. La escala es adecuada en general. El manejo de la topografía es funcional (cumple con niveles) pero carece de una intención poética o de integración profunda con el código.</t>
+          <t>Las 5 propuestas demuestran una exploración morfológica arriesgada y diversa. El manejo de la escala es impecable. La propuesta integra la topografía del lote de forma creativa, convirtiendo la pendiente en una oportunidad proyectual.</t>
         </is>
       </c>
       <c r="H438" t="inlineStr">
@@ -21879,7 +21879,7 @@
       </c>
       <c r="C462" t="inlineStr">
         <is>
-          <t>4.1</t>
+          <t>4.3</t>
         </is>
       </c>
       <c r="D462" t="inlineStr">
@@ -21898,7 +21898,7 @@
         </is>
       </c>
       <c r="G462" t="n">
-        <v>4.053571428571429</v>
+        <v>4.303571428571429</v>
       </c>
       <c r="H462" t="inlineStr">
         <is>
@@ -21922,7 +21922,7 @@
       </c>
       <c r="C463" t="inlineStr">
         <is>
-          <t>4.0</t>
+          <t>5.0</t>
         </is>
       </c>
       <c r="D463" t="inlineStr">
@@ -23026,12 +23026,12 @@
       </c>
       <c r="C487" t="inlineStr">
         <is>
-          <t>3.6</t>
+          <t>4.7</t>
         </is>
       </c>
       <c r="D487" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="E487" t="inlineStr">
@@ -23041,11 +23041,11 @@
       </c>
       <c r="F487" t="inlineStr">
         <is>
-          <t>E3.Coment_B</t>
+          <t>E3.Coment_A</t>
         </is>
       </c>
       <c r="G487" t="n">
-        <v>3.593928571428571</v>
+        <v>4.677678571428571</v>
       </c>
       <c r="H487" t="inlineStr">
         <is>
@@ -23071,12 +23071,12 @@
       </c>
       <c r="C488" t="inlineStr">
         <is>
-          <t>2.8</t>
+          <t>4.7</t>
         </is>
       </c>
       <c r="D488" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>A</t>
         </is>
       </c>
       <c r="E488" t="inlineStr">
@@ -23086,12 +23086,12 @@
       </c>
       <c r="F488" t="inlineStr">
         <is>
-          <t>E3.Func_C</t>
+          <t>E3.Func_A</t>
         </is>
       </c>
       <c r="G488" t="inlineStr">
         <is>
-          <t>Escasa diversidad formal. Errores críticos de escala. La propuesta ignora la topografía o se limita a soluciones genéricas (ej. aplanamiento masivo) sin diálogo con el terreno.</t>
+          <t>Las 5 propuestas demuestran una exploración morfológica arriesgada y diversa. El manejo de la escala es impecable. La propuesta integra la topografía del lote de forma creativa, convirtiendo la pendiente en una oportunidad proyectual.</t>
         </is>
       </c>
       <c r="H488" t="inlineStr">
@@ -23118,12 +23118,12 @@
       </c>
       <c r="C489" t="inlineStr">
         <is>
-          <t>2.2</t>
+          <t>4.2</t>
         </is>
       </c>
       <c r="D489" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>A</t>
         </is>
       </c>
       <c r="E489" t="inlineStr">
@@ -23133,12 +23133,12 @@
       </c>
       <c r="F489" t="inlineStr">
         <is>
-          <t>E3.Rep_C</t>
+          <t>E3.Rep_A</t>
         </is>
       </c>
       <c r="G489" t="inlineStr">
         <is>
-          <t>Planimetría confusa, incompleta o sin rigor técnico (falta de escala gráfica/numérica, linderos ausentes). Las maquetas son precarias y no permiten entender la espacialidad propuesta.</t>
+          <t>La planimetría (plantas 1:100) es clara, técnica y expresiva; incluye cotas, amoblamiento y una relación clara con el contexto/lote. Las maquetas volumétricas poseen una factura impecable y tienen relación directa con la planimetría correspondiente</t>
         </is>
       </c>
       <c r="H489" t="inlineStr">
@@ -23165,7 +23165,7 @@
       </c>
       <c r="C490" t="inlineStr">
         <is>
-          <t>4.3</t>
+          <t>4.8</t>
         </is>
       </c>
       <c r="D490" t="inlineStr">
@@ -24202,12 +24202,12 @@
       </c>
       <c r="C512" t="inlineStr">
         <is>
-          <t>0.6</t>
+          <t>4.4</t>
         </is>
       </c>
       <c r="D512" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>A</t>
         </is>
       </c>
       <c r="E512" t="inlineStr">
@@ -24217,11 +24217,11 @@
       </c>
       <c r="F512" t="inlineStr">
         <is>
-          <t>E3.Coment_C</t>
+          <t>E3.Coment_A</t>
         </is>
       </c>
       <c r="G512" t="n">
-        <v>0.625</v>
+        <v>4.375</v>
       </c>
       <c r="H512" t="inlineStr">
         <is>
@@ -24247,12 +24247,12 @@
       </c>
       <c r="C513" t="inlineStr">
         <is>
-          <t>0.0</t>
+          <t>5.0</t>
         </is>
       </c>
       <c r="D513" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>A</t>
         </is>
       </c>
       <c r="E513" t="inlineStr">
@@ -24262,12 +24262,12 @@
       </c>
       <c r="F513" t="inlineStr">
         <is>
-          <t>E3.Func_C</t>
+          <t>E3.Func_A</t>
         </is>
       </c>
       <c r="G513" t="inlineStr">
         <is>
-          <t>Escasa diversidad formal. Errores críticos de escala. La propuesta ignora la topografía o se limita a soluciones genéricas (ej. aplanamiento masivo) sin diálogo con el terreno.</t>
+          <t>Las 5 propuestas demuestran una exploración morfológica arriesgada y diversa. El manejo de la escala es impecable. La propuesta integra la topografía del lote de forma creativa, convirtiendo la pendiente en una oportunidad proyectual.</t>
         </is>
       </c>
       <c r="H513" t="inlineStr">
@@ -24294,12 +24294,12 @@
       </c>
       <c r="C514" t="inlineStr">
         <is>
-          <t>0.0</t>
+          <t>5.0</t>
         </is>
       </c>
       <c r="D514" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>A</t>
         </is>
       </c>
       <c r="E514" t="inlineStr">
@@ -24309,12 +24309,12 @@
       </c>
       <c r="F514" t="inlineStr">
         <is>
-          <t>E3.Rep_C</t>
+          <t>E3.Rep_A</t>
         </is>
       </c>
       <c r="G514" t="inlineStr">
         <is>
-          <t>Planimetría confusa, incompleta o sin rigor técnico (falta de escala gráfica/numérica, linderos ausentes). Las maquetas son precarias y no permiten entender la espacialidad propuesta.</t>
+          <t>La planimetría (plantas 1:100) es clara, técnica y expresiva; incluye cotas, amoblamiento y una relación clara con el contexto/lote. Las maquetas volumétricas poseen una factura impecable y tienen relación directa con la planimetría correspondiente</t>
         </is>
       </c>
       <c r="H514" t="inlineStr">
@@ -24341,12 +24341,12 @@
       </c>
       <c r="C515" t="inlineStr">
         <is>
-          <t>0.0</t>
+          <t>5.0</t>
         </is>
       </c>
       <c r="D515" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>A</t>
         </is>
       </c>
       <c r="E515" t="inlineStr">
@@ -24356,12 +24356,12 @@
       </c>
       <c r="F515" t="inlineStr">
         <is>
-          <t>E3.Arg_C</t>
+          <t>E3.Arg_A</t>
         </is>
       </c>
       <c r="G515" t="inlineStr">
         <is>
-          <t>La bitácora se presenta como un requisito administrativo y no como una herramienta de diseño. No hay coherencia entre el programa construido y las plantas presentadas. Faltan varios productos esenciales de la entrega.</t>
+          <t>Existe una trazabilidad absoluta entre el proceso en bitácora (árbol de convivencia, línea de tiempo, tabla de acciones y código) y las 5 ideas finales. Entrega la totalidad de los productos solicitados.</t>
         </is>
       </c>
       <c r="H515" t="inlineStr">
@@ -25377,7 +25377,7 @@
       </c>
       <c r="C537" t="inlineStr">
         <is>
-          <t>4.8</t>
+          <t>5.0</t>
         </is>
       </c>
       <c r="D537" t="inlineStr">
@@ -25396,7 +25396,7 @@
         </is>
       </c>
       <c r="G537" t="n">
-        <v>4.75</v>
+        <v>5</v>
       </c>
       <c r="H537" t="inlineStr">
         <is>
@@ -25422,7 +25422,7 @@
       </c>
       <c r="C538" t="inlineStr">
         <is>
-          <t>4.0</t>
+          <t>5.0</t>
         </is>
       </c>
       <c r="D538" t="inlineStr">
@@ -26553,7 +26553,7 @@
       </c>
       <c r="C562" t="inlineStr">
         <is>
-          <t>4.2</t>
+          <t>4.3</t>
         </is>
       </c>
       <c r="D562" t="inlineStr">
@@ -26572,7 +26572,7 @@
         </is>
       </c>
       <c r="G562" t="n">
-        <v>4.1625</v>
+        <v>4.34375</v>
       </c>
       <c r="H562" t="inlineStr">
         <is>
@@ -26598,12 +26598,12 @@
       </c>
       <c r="C563" t="inlineStr">
         <is>
-          <t>2.9</t>
+          <t>3.6</t>
         </is>
       </c>
       <c r="D563" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>B</t>
         </is>
       </c>
       <c r="E563" t="inlineStr">
@@ -26613,12 +26613,12 @@
       </c>
       <c r="F563" t="inlineStr">
         <is>
-          <t>E3.Func_C</t>
+          <t>E3.Func_B</t>
         </is>
       </c>
       <c r="G563" t="inlineStr">
         <is>
-          <t>Escasa diversidad formal. Errores críticos de escala. La propuesta ignora la topografía o se limita a soluciones genéricas (ej. aplanamiento masivo) sin diálogo con el terreno.</t>
+          <t>Existe exploración morfológica pero con menor toma de riesgos. La escala es adecuada en general. El manejo de la topografía es funcional (cumple con niveles) pero carece de una intención poética o de integración profunda con el código.</t>
         </is>
       </c>
       <c r="H563" t="inlineStr">
@@ -27728,7 +27728,7 @@
       </c>
       <c r="C587" t="inlineStr">
         <is>
-          <t>4.7</t>
+          <t>5.0</t>
         </is>
       </c>
       <c r="D587" t="inlineStr">
@@ -27747,7 +27747,7 @@
         </is>
       </c>
       <c r="G587" t="n">
-        <v>4.71</v>
+        <v>4.95</v>
       </c>
       <c r="H587" t="inlineStr">
         <is>
@@ -27773,12 +27773,12 @@
       </c>
       <c r="C588" t="inlineStr">
         <is>
-          <t>3.8</t>
+          <t>4.8</t>
         </is>
       </c>
       <c r="D588" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="E588" t="inlineStr">
@@ -27788,12 +27788,12 @@
       </c>
       <c r="F588" t="inlineStr">
         <is>
-          <t>E3.Func_B</t>
+          <t>E3.Func_A</t>
         </is>
       </c>
       <c r="G588" t="inlineStr">
         <is>
-          <t>Existe exploración morfológica pero con menor toma de riesgos. La escala es adecuada en general. El manejo de la topografía es funcional (cumple con niveles) pero carece de una intención poética o de integración profunda con el código.</t>
+          <t>Las 5 propuestas demuestran una exploración morfológica arriesgada y diversa. El manejo de la escala es impecable. La propuesta integra la topografía del lote de forma creativa, convirtiendo la pendiente en una oportunidad proyectual.</t>
         </is>
       </c>
       <c r="H588" t="inlineStr">
@@ -28901,7 +28901,7 @@
       </c>
       <c r="C612" t="inlineStr">
         <is>
-          <t>4.7</t>
+          <t>4.9</t>
         </is>
       </c>
       <c r="D612" t="inlineStr">
@@ -28920,7 +28920,7 @@
         </is>
       </c>
       <c r="G612" t="n">
-        <v>4.663571428571428</v>
+        <v>4.945535714285715</v>
       </c>
       <c r="H612" t="inlineStr">
         <is>
@@ -28946,12 +28946,12 @@
       </c>
       <c r="C613" t="inlineStr">
         <is>
-          <t>3.9</t>
+          <t>4.9</t>
         </is>
       </c>
       <c r="D613" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="E613" t="inlineStr">
@@ -28961,12 +28961,12 @@
       </c>
       <c r="F613" t="inlineStr">
         <is>
-          <t>E3.Func_B</t>
+          <t>E3.Func_A</t>
         </is>
       </c>
       <c r="G613" t="inlineStr">
         <is>
-          <t>Existe exploración morfológica pero con menor toma de riesgos. La escala es adecuada en general. El manejo de la topografía es funcional (cumple con niveles) pero carece de una intención poética o de integración profunda con el código.</t>
+          <t>Las 5 propuestas demuestran una exploración morfológica arriesgada y diversa. El manejo de la escala es impecable. La propuesta integra la topografía del lote de forma creativa, convirtiendo la pendiente en una oportunidad proyectual.</t>
         </is>
       </c>
       <c r="H613" t="inlineStr">
@@ -29040,7 +29040,7 @@
       </c>
       <c r="C615" t="inlineStr">
         <is>
-          <t>4.7</t>
+          <t>4.9</t>
         </is>
       </c>
       <c r="D615" t="inlineStr">
@@ -30074,7 +30074,7 @@
       </c>
       <c r="C637" t="inlineStr">
         <is>
-          <t>0.6</t>
+          <t>2.4</t>
         </is>
       </c>
       <c r="D637" t="inlineStr">
@@ -30093,7 +30093,7 @@
         </is>
       </c>
       <c r="G637" t="n">
-        <v>0.625</v>
+        <v>2.375</v>
       </c>
       <c r="H637" t="inlineStr">
         <is>
@@ -30119,12 +30119,12 @@
       </c>
       <c r="C638" t="inlineStr">
         <is>
-          <t>0.0</t>
+          <t>5.0</t>
         </is>
       </c>
       <c r="D638" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>A</t>
         </is>
       </c>
       <c r="E638" t="inlineStr">
@@ -30134,12 +30134,12 @@
       </c>
       <c r="F638" t="inlineStr">
         <is>
-          <t>E3.Func_C</t>
+          <t>E3.Func_A</t>
         </is>
       </c>
       <c r="G638" t="inlineStr">
         <is>
-          <t>Escasa diversidad formal. Errores críticos de escala. La propuesta ignora la topografía o se limita a soluciones genéricas (ej. aplanamiento masivo) sin diálogo con el terreno.</t>
+          <t>Las 5 propuestas demuestran una exploración morfológica arriesgada y diversa. El manejo de la escala es impecable. La propuesta integra la topografía del lote de forma creativa, convirtiendo la pendiente en una oportunidad proyectual.</t>
         </is>
       </c>
       <c r="H638" t="inlineStr">
@@ -30166,12 +30166,12 @@
       </c>
       <c r="C639" t="inlineStr">
         <is>
-          <t>0.0</t>
+          <t>5.0</t>
         </is>
       </c>
       <c r="D639" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>A</t>
         </is>
       </c>
       <c r="E639" t="inlineStr">
@@ -30181,12 +30181,12 @@
       </c>
       <c r="F639" t="inlineStr">
         <is>
-          <t>E3.Rep_C</t>
+          <t>E3.Rep_A</t>
         </is>
       </c>
       <c r="G639" t="inlineStr">
         <is>
-          <t>Planimetría confusa, incompleta o sin rigor técnico (falta de escala gráfica/numérica, linderos ausentes). Las maquetas son precarias y no permiten entender la espacialidad propuesta.</t>
+          <t>La planimetría (plantas 1:100) es clara, técnica y expresiva; incluye cotas, amoblamiento y una relación clara con el contexto/lote. Las maquetas volumétricas poseen una factura impecable y tienen relación directa con la planimetría correspondiente</t>
         </is>
       </c>
       <c r="H639" t="inlineStr">
@@ -30213,12 +30213,12 @@
       </c>
       <c r="C640" t="inlineStr">
         <is>
-          <t>0.0</t>
+          <t>5.0</t>
         </is>
       </c>
       <c r="D640" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>A</t>
         </is>
       </c>
       <c r="E640" t="inlineStr">
@@ -30228,12 +30228,12 @@
       </c>
       <c r="F640" t="inlineStr">
         <is>
-          <t>E3.Arg_C</t>
+          <t>E3.Arg_A</t>
         </is>
       </c>
       <c r="G640" t="inlineStr">
         <is>
-          <t>La bitácora se presenta como un requisito administrativo y no como una herramienta de diseño. No hay coherencia entre el programa construido y las plantas presentadas. Faltan varios productos esenciales de la entrega.</t>
+          <t>Existe una trazabilidad absoluta entre el proceso en bitácora (árbol de convivencia, línea de tiempo, tabla de acciones y código) y las 5 ideas finales. Entrega la totalidad de los productos solicitados.</t>
         </is>
       </c>
       <c r="H640" t="inlineStr">
@@ -31248,7 +31248,7 @@
       </c>
       <c r="C662" t="inlineStr">
         <is>
-          <t>4.7</t>
+          <t>4.9</t>
         </is>
       </c>
       <c r="D662" t="inlineStr">
@@ -31267,7 +31267,7 @@
         </is>
       </c>
       <c r="G662" t="n">
-        <v>4.6625</v>
+        <v>4.90625</v>
       </c>
       <c r="H662" t="inlineStr">
         <is>
@@ -31293,12 +31293,12 @@
       </c>
       <c r="C663" t="inlineStr">
         <is>
-          <t>3.9</t>
+          <t>4.9</t>
         </is>
       </c>
       <c r="D663" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="E663" t="inlineStr">
@@ -31308,12 +31308,12 @@
       </c>
       <c r="F663" t="inlineStr">
         <is>
-          <t>E3.Func_B</t>
+          <t>E3.Func_A</t>
         </is>
       </c>
       <c r="G663" t="inlineStr">
         <is>
-          <t>Existe exploración morfológica pero con menor toma de riesgos. La escala es adecuada en general. El manejo de la topografía es funcional (cumple con niveles) pero carece de una intención poética o de integración profunda con el código.</t>
+          <t>Las 5 propuestas demuestran una exploración morfológica arriesgada y diversa. El manejo de la escala es impecable. La propuesta integra la topografía del lote de forma creativa, convirtiendo la pendiente en una oportunidad proyectual.</t>
         </is>
       </c>
       <c r="H663" t="inlineStr">
@@ -32425,7 +32425,7 @@
       </c>
       <c r="C687" t="inlineStr">
         <is>
-          <t>4.6</t>
+          <t>4.9</t>
         </is>
       </c>
       <c r="D687" t="inlineStr">
@@ -32444,7 +32444,7 @@
         </is>
       </c>
       <c r="G687" t="n">
-        <v>4.6475</v>
+        <v>4.8875</v>
       </c>
       <c r="H687" t="inlineStr">
         <is>
@@ -32470,12 +32470,12 @@
       </c>
       <c r="C688" t="inlineStr">
         <is>
-          <t>3.8</t>
+          <t>4.8</t>
         </is>
       </c>
       <c r="D688" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="E688" t="inlineStr">
@@ -32485,12 +32485,12 @@
       </c>
       <c r="F688" t="inlineStr">
         <is>
-          <t>E3.Func_B</t>
+          <t>E3.Func_A</t>
         </is>
       </c>
       <c r="G688" t="inlineStr">
         <is>
-          <t>Existe exploración morfológica pero con menor toma de riesgos. La escala es adecuada en general. El manejo de la topografía es funcional (cumple con niveles) pero carece de una intención poética o de integración profunda con el código.</t>
+          <t>Las 5 propuestas demuestran una exploración morfológica arriesgada y diversa. El manejo de la escala es impecable. La propuesta integra la topografía del lote de forma creativa, convirtiendo la pendiente en una oportunidad proyectual.</t>
         </is>
       </c>
       <c r="H688" t="inlineStr">
@@ -33597,7 +33597,7 @@
       </c>
       <c r="C712" t="inlineStr">
         <is>
-          <t>4.7</t>
+          <t>4.9</t>
         </is>
       </c>
       <c r="D712" t="inlineStr">
@@ -33616,7 +33616,7 @@
         </is>
       </c>
       <c r="G712" t="n">
-        <v>4.6875</v>
+        <v>4.9375</v>
       </c>
       <c r="H712" t="inlineStr">
         <is>
@@ -33642,7 +33642,7 @@
       </c>
       <c r="C713" t="inlineStr">
         <is>
-          <t>4.0</t>
+          <t>5.0</t>
         </is>
       </c>
       <c r="D713" t="inlineStr">
@@ -34773,12 +34773,12 @@
       </c>
       <c r="C737" t="inlineStr">
         <is>
-          <t>0.6</t>
+          <t>4.0</t>
         </is>
       </c>
       <c r="D737" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>A</t>
         </is>
       </c>
       <c r="E737" t="inlineStr">
@@ -34788,11 +34788,11 @@
       </c>
       <c r="F737" t="inlineStr">
         <is>
-          <t>E3.Coment_C</t>
+          <t>E3.Coment_A</t>
         </is>
       </c>
       <c r="G737" t="n">
-        <v>0.625</v>
+        <v>4.00625</v>
       </c>
       <c r="H737" t="inlineStr">
         <is>
@@ -34818,12 +34818,12 @@
       </c>
       <c r="C738" t="inlineStr">
         <is>
-          <t>0.0</t>
+          <t>4.6</t>
         </is>
       </c>
       <c r="D738" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>A</t>
         </is>
       </c>
       <c r="E738" t="inlineStr">
@@ -34833,12 +34833,12 @@
       </c>
       <c r="F738" t="inlineStr">
         <is>
-          <t>E3.Func_C</t>
+          <t>E3.Func_A</t>
         </is>
       </c>
       <c r="G738" t="inlineStr">
         <is>
-          <t>Escasa diversidad formal. Errores críticos de escala. La propuesta ignora la topografía o se limita a soluciones genéricas (ej. aplanamiento masivo) sin diálogo con el terreno.</t>
+          <t>Las 5 propuestas demuestran una exploración morfológica arriesgada y diversa. El manejo de la escala es impecable. La propuesta integra la topografía del lote de forma creativa, convirtiendo la pendiente en una oportunidad proyectual.</t>
         </is>
       </c>
       <c r="H738" t="inlineStr">
@@ -34865,12 +34865,12 @@
       </c>
       <c r="C739" t="inlineStr">
         <is>
-          <t>0.0</t>
+          <t>3.9</t>
         </is>
       </c>
       <c r="D739" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>B</t>
         </is>
       </c>
       <c r="E739" t="inlineStr">
@@ -34880,12 +34880,12 @@
       </c>
       <c r="F739" t="inlineStr">
         <is>
-          <t>E3.Rep_C</t>
+          <t>E3.Rep_B</t>
         </is>
       </c>
       <c r="G739" t="inlineStr">
         <is>
-          <t>Planimetría confusa, incompleta o sin rigor técnico (falta de escala gráfica/numérica, linderos ausentes). Las maquetas son precarias y no permiten entender la espacialidad propuesta.</t>
+          <t>La representación técnica es legible pero carece de detalles esenciales (ej. falta de cotas o amoblamiento genérico que no explica el uso). La factura de las maquetas es aceptable, aunque se observan descuidos en la limpieza o su relación con la planimetría correspondiente</t>
         </is>
       </c>
       <c r="H739" t="inlineStr">
@@ -34912,12 +34912,12 @@
       </c>
       <c r="C740" t="inlineStr">
         <is>
-          <t>0.0</t>
+          <t>5.0</t>
         </is>
       </c>
       <c r="D740" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>A</t>
         </is>
       </c>
       <c r="E740" t="inlineStr">
@@ -34927,12 +34927,12 @@
       </c>
       <c r="F740" t="inlineStr">
         <is>
-          <t>E3.Arg_C</t>
+          <t>E3.Arg_A</t>
         </is>
       </c>
       <c r="G740" t="inlineStr">
         <is>
-          <t>La bitácora se presenta como un requisito administrativo y no como una herramienta de diseño. No hay coherencia entre el programa construido y las plantas presentadas. Faltan varios productos esenciales de la entrega.</t>
+          <t>Existe una trazabilidad absoluta entre el proceso en bitácora (árbol de convivencia, línea de tiempo, tabla de acciones y código) y las 5 ideas finales. Entrega la totalidad de los productos solicitados.</t>
         </is>
       </c>
       <c r="H740" t="inlineStr">
@@ -35948,12 +35948,12 @@
       </c>
       <c r="C762" t="inlineStr">
         <is>
-          <t>3.8</t>
+          <t>4.3</t>
         </is>
       </c>
       <c r="D762" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="E762" t="inlineStr">
@@ -35963,11 +35963,11 @@
       </c>
       <c r="F762" t="inlineStr">
         <is>
-          <t>E3.Coment_B</t>
+          <t>E3.Coment_A</t>
         </is>
       </c>
       <c r="G762" t="n">
-        <v>3.788571428571428</v>
+        <v>4.297321428571428</v>
       </c>
       <c r="H762" t="inlineStr">
         <is>
@@ -35993,12 +35993,12 @@
       </c>
       <c r="C763" t="inlineStr">
         <is>
-          <t>2.6</t>
+          <t>4.2</t>
         </is>
       </c>
       <c r="D763" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>A</t>
         </is>
       </c>
       <c r="E763" t="inlineStr">
@@ -36008,12 +36008,12 @@
       </c>
       <c r="F763" t="inlineStr">
         <is>
-          <t>E3.Func_C</t>
+          <t>E3.Func_A</t>
         </is>
       </c>
       <c r="G763" t="inlineStr">
         <is>
-          <t>Escasa diversidad formal. Errores críticos de escala. La propuesta ignora la topografía o se limita a soluciones genéricas (ej. aplanamiento masivo) sin diálogo con el terreno.</t>
+          <t>Las 5 propuestas demuestran una exploración morfológica arriesgada y diversa. El manejo de la escala es impecable. La propuesta integra la topografía del lote de forma creativa, convirtiendo la pendiente en una oportunidad proyectual.</t>
         </is>
       </c>
       <c r="H763" t="inlineStr">
@@ -36087,12 +36087,12 @@
       </c>
       <c r="C765" t="inlineStr">
         <is>
-          <t>3.7</t>
+          <t>4.2</t>
         </is>
       </c>
       <c r="D765" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="E765" t="inlineStr">
@@ -36102,12 +36102,12 @@
       </c>
       <c r="F765" t="inlineStr">
         <is>
-          <t>E3.Arg_B</t>
+          <t>E3.Arg_A</t>
         </is>
       </c>
       <c r="G765" t="inlineStr">
         <is>
-          <t>La bitácora contiene los elementos solicitados, pero el vínculo entre el análisis (árbol, línea del tiempo, tabla y código) y las propuestas finales se siente forzado o desconectado. Hacen falta algunos productos.</t>
+          <t>Existe una trazabilidad absoluta entre el proceso en bitácora (árbol de convivencia, línea de tiempo, tabla de acciones y código) y las 5 ideas finales. Entrega la totalidad de los productos solicitados.</t>
         </is>
       </c>
       <c r="H765" t="inlineStr">

</xml_diff>